<commit_message>
feat: setup interactive portfolio and Quartz notes vault
</commit_message>
<xml_diff>
--- a/Relative Valuation/Relative valuation Pharma industry.xlsx
+++ b/Relative Valuation/Relative valuation Pharma industry.xlsx
@@ -5,16 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\FP&amp;A Practice\Relative Valuation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\FP&amp;A Practice\Equity-Research-Models\Relative Valuation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E6A6BC-32CE-4CDC-8775-0B60B3A6BC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01624A22-2E5E-4BDA-A798-0696D5763FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{D574B39C-01AB-49CD-9EEF-5F61B89E5F63}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D574B39C-01AB-49CD-9EEF-5F61B89E5F63}"/>
   </bookViews>
   <sheets>
     <sheet name="PHARMA" sheetId="1" r:id="rId1"/>
-    <sheet name="BANKING" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
   <si>
     <t>Implied Value Per Share</t>
   </si>
@@ -157,45 +156,6 @@
   </si>
   <si>
     <t>Relative Valuation method 24/03/26 Healthcare</t>
-  </si>
-  <si>
-    <t>Relative Valuation method 4/05/26 Banking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axis Bank </t>
-  </si>
-  <si>
-    <t>SBI Bank</t>
-  </si>
-  <si>
-    <t>HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICICI </t>
-  </si>
-  <si>
-    <t>Kotak Mahindra</t>
-  </si>
-  <si>
-    <t>Indusind</t>
-  </si>
-  <si>
-    <t>AXISBANK</t>
-  </si>
-  <si>
-    <t>SBIN</t>
-  </si>
-  <si>
-    <t>HDFCBANK</t>
-  </si>
-  <si>
-    <t>ICICIBANK</t>
-  </si>
-  <si>
-    <t>KOTAKBANK</t>
-  </si>
-  <si>
-    <t>INDUSINDBK</t>
   </si>
 </sst>
 </file>
@@ -445,27 +405,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1452,758 +1392,6 @@
     <mergeCell ref="N4:P4"/>
   </mergeCells>
   <conditionalFormatting sqref="N27:P27">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Overvalued">
-      <formula>NOT(ISERROR(SEARCH("Overvalued",N27)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Undervalued">
-      <formula>NOT(ISERROR(SEARCH("Undervalued",N27)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D62924-870C-4A1B-8419-A62243E43A45}">
-  <dimension ref="B2:Q27"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="8.09765625" customWidth="1"/>
-    <col min="2" max="2" width="16.69921875" customWidth="1"/>
-    <col min="3" max="3" width="11.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.59765625" customWidth="1"/>
-    <col min="6" max="6" width="10.09765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.796875" customWidth="1"/>
-    <col min="10" max="10" width="8.09765625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.19921875" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.59765625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:16" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B2" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-    </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="K4" s="50"/>
-      <c r="L4" s="50"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="O4" s="50"/>
-      <c r="P4" s="50"/>
-    </row>
-    <row r="5" spans="2:16" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B5" s="44" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="43" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" s="43" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="I5" s="10"/>
-      <c r="J5" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="K5" s="42" t="s">
-        <v>28</v>
-      </c>
-      <c r="L5" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="M5" s="42"/>
-      <c r="N5" s="42" t="s">
-        <v>8</v>
-      </c>
-      <c r="O5" s="42" t="s">
-        <v>7</v>
-      </c>
-      <c r="P5" s="42" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="39"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="39"/>
-      <c r="L6" s="39"/>
-      <c r="M6" s="39"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="39"/>
-      <c r="P6" s="39"/>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B7" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="36">
-        <v>1275</v>
-      </c>
-      <c r="E7" s="33">
-        <v>310</v>
-      </c>
-      <c r="F7" s="34">
-        <f t="shared" ref="F7:F12" si="0">D7*E7</f>
-        <v>395250</v>
-      </c>
-      <c r="G7" s="35">
-        <f>3275-1099</f>
-        <v>2176</v>
-      </c>
-      <c r="H7" s="34">
-        <f t="shared" ref="H7:H12" si="1">F7+G7</f>
-        <v>397426</v>
-      </c>
-      <c r="I7" s="33"/>
-      <c r="J7" s="33">
-        <v>8140</v>
-      </c>
-      <c r="K7" s="33">
-        <v>2319</v>
-      </c>
-      <c r="L7" s="33">
-        <v>1419</v>
-      </c>
-      <c r="M7" s="32"/>
-      <c r="N7" s="31">
-        <f t="shared" ref="N7:N12" si="2">H7/J7</f>
-        <v>48.823832923832924</v>
-      </c>
-      <c r="O7" s="31">
-        <f t="shared" ref="O7:O12" si="3">H7/K7</f>
-        <v>171.37818025010782</v>
-      </c>
-      <c r="P7" s="31">
-        <f t="shared" ref="P7:P12" si="4">F7/L7</f>
-        <v>278.54122621564483</v>
-      </c>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B8" s="30" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="28">
-        <v>1068</v>
-      </c>
-      <c r="E8" s="25">
-        <v>892</v>
-      </c>
-      <c r="F8" s="20">
-        <f t="shared" si="0"/>
-        <v>952656</v>
-      </c>
-      <c r="G8" s="27">
-        <f>7987-934</f>
-        <v>7053</v>
-      </c>
-      <c r="H8" s="20">
-        <f t="shared" si="1"/>
-        <v>959709</v>
-      </c>
-      <c r="I8" s="26"/>
-      <c r="J8" s="25">
-        <v>24125</v>
-      </c>
-      <c r="K8" s="25">
-        <v>3022</v>
-      </c>
-      <c r="L8" s="25">
-        <v>1866</v>
-      </c>
-      <c r="M8" s="20"/>
-      <c r="N8" s="17">
-        <f t="shared" si="2"/>
-        <v>39.780683937823831</v>
-      </c>
-      <c r="O8" s="17">
-        <f t="shared" si="3"/>
-        <v>317.57412309728659</v>
-      </c>
-      <c r="P8" s="17">
-        <f t="shared" si="4"/>
-        <v>510.53376205787782</v>
-      </c>
-    </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B9" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="22">
-        <v>779</v>
-      </c>
-      <c r="E9" s="19">
-        <v>1530</v>
-      </c>
-      <c r="F9" s="20">
-        <f t="shared" si="0"/>
-        <v>1191870</v>
-      </c>
-      <c r="G9" s="21">
-        <f>3195-598</f>
-        <v>2597</v>
-      </c>
-      <c r="H9" s="20">
-        <f t="shared" si="1"/>
-        <v>1194467</v>
-      </c>
-      <c r="I9" s="1"/>
-      <c r="J9" s="19">
-        <v>8770</v>
-      </c>
-      <c r="K9" s="19">
-        <v>1655</v>
-      </c>
-      <c r="L9" s="19">
-        <v>981</v>
-      </c>
-      <c r="M9" s="18"/>
-      <c r="N9" s="17">
-        <f t="shared" si="2"/>
-        <v>136.19920182440137</v>
-      </c>
-      <c r="O9" s="17">
-        <f t="shared" si="3"/>
-        <v>721.73232628398796</v>
-      </c>
-      <c r="P9" s="17">
-        <f t="shared" si="4"/>
-        <v>1214.954128440367</v>
-      </c>
-    </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B10" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="22">
-        <v>1271</v>
-      </c>
-      <c r="E10" s="19">
-        <v>712</v>
-      </c>
-      <c r="F10" s="20">
-        <f t="shared" si="0"/>
-        <v>904952</v>
-      </c>
-      <c r="G10" s="21">
-        <f>2050284-113747</f>
-        <v>1936537</v>
-      </c>
-      <c r="H10" s="20">
-        <f t="shared" si="1"/>
-        <v>2841489</v>
-      </c>
-      <c r="I10" s="1"/>
-      <c r="J10" s="19">
-        <v>6778</v>
-      </c>
-      <c r="K10" s="19">
-        <v>1368.4</v>
-      </c>
-      <c r="L10" s="19">
-        <v>779</v>
-      </c>
-      <c r="M10" s="18"/>
-      <c r="N10" s="17">
-        <f t="shared" si="2"/>
-        <v>419.22233697255825</v>
-      </c>
-      <c r="O10" s="17">
-        <f t="shared" si="3"/>
-        <v>2076.5046769950304</v>
-      </c>
-      <c r="P10" s="17">
-        <f t="shared" si="4"/>
-        <v>1161.6842105263158</v>
-      </c>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B11" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="22">
-        <v>372</v>
-      </c>
-      <c r="E11" s="19">
-        <v>994</v>
-      </c>
-      <c r="F11" s="20">
-        <f t="shared" si="0"/>
-        <v>369768</v>
-      </c>
-      <c r="G11" s="21">
-        <f>662334-40006</f>
-        <v>622328</v>
-      </c>
-      <c r="H11" s="20">
-        <f t="shared" si="1"/>
-        <v>992096</v>
-      </c>
-      <c r="I11" s="1"/>
-      <c r="J11" s="19">
-        <v>4461</v>
-      </c>
-      <c r="K11" s="19">
-        <v>1661</v>
-      </c>
-      <c r="L11" s="19">
-        <v>359</v>
-      </c>
-      <c r="M11" s="18"/>
-      <c r="N11" s="17">
-        <f t="shared" si="2"/>
-        <v>222.39318538444294</v>
-      </c>
-      <c r="O11" s="17">
-        <f t="shared" si="3"/>
-        <v>597.28838049367846</v>
-      </c>
-      <c r="P11" s="17">
-        <f t="shared" si="4"/>
-        <v>1029.9944289693594</v>
-      </c>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B12" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="22">
-        <v>914</v>
-      </c>
-      <c r="E12" s="19">
-        <v>78</v>
-      </c>
-      <c r="F12" s="20">
-        <f t="shared" si="0"/>
-        <v>71292</v>
-      </c>
-      <c r="G12" s="21">
-        <f>442720-49711</f>
-        <v>393009</v>
-      </c>
-      <c r="H12" s="20">
-        <f t="shared" si="1"/>
-        <v>464301</v>
-      </c>
-      <c r="I12" s="1"/>
-      <c r="J12" s="19">
-        <v>4182</v>
-      </c>
-      <c r="K12" s="19">
-        <v>956.2</v>
-      </c>
-      <c r="L12" s="19">
-        <v>514</v>
-      </c>
-      <c r="M12" s="18"/>
-      <c r="N12" s="17">
-        <f t="shared" si="2"/>
-        <v>111.02367288378767</v>
-      </c>
-      <c r="O12" s="17">
-        <f t="shared" si="3"/>
-        <v>485.56891863626856</v>
-      </c>
-      <c r="P12" s="17">
-        <f t="shared" si="4"/>
-        <v>138.70038910505838</v>
-      </c>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="E13" s="8"/>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B14" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="14"/>
-      <c r="N14" s="13">
-        <f>MAX(N8:N12)</f>
-        <v>419.22233697255825</v>
-      </c>
-      <c r="O14" s="13">
-        <f>MAX(O8:O12)</f>
-        <v>2076.5046769950304</v>
-      </c>
-      <c r="P14" s="13">
-        <f>MAX(P8:P12)</f>
-        <v>1214.954128440367</v>
-      </c>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B15" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="13">
-        <f>QUARTILE(N8:N12,3)</f>
-        <v>222.39318538444294</v>
-      </c>
-      <c r="O15" s="13">
-        <f>QUARTILE(O8:O12,3)</f>
-        <v>721.73232628398796</v>
-      </c>
-      <c r="P15" s="13">
-        <f>QUARTILE(P8:P12,3)</f>
-        <v>1161.6842105263158</v>
-      </c>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B16" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
-      <c r="N16" s="16">
-        <f>AVERAGE(N8:N12)</f>
-        <v>185.72381620060281</v>
-      </c>
-      <c r="O16" s="16">
-        <f>AVERAGE(O8:O12)</f>
-        <v>839.73368510125033</v>
-      </c>
-      <c r="P16" s="16">
-        <f>AVERAGE(P8:P12)</f>
-        <v>811.17338381979573</v>
-      </c>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B17" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15"/>
-      <c r="N17" s="16">
-        <f>MEDIAN(N8:N12)</f>
-        <v>136.19920182440137</v>
-      </c>
-      <c r="O17" s="16">
-        <f>MEDIAN(O8:O12)</f>
-        <v>597.28838049367846</v>
-      </c>
-      <c r="P17" s="16">
-        <f>MEDIAN(P8:P12)</f>
-        <v>1029.9944289693594</v>
-      </c>
-    </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B18" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="13">
-        <f>QUARTILE(N8:N12,1)</f>
-        <v>111.02367288378767</v>
-      </c>
-      <c r="O18" s="13">
-        <f>QUARTILE(O8:O12,1)</f>
-        <v>485.56891863626856</v>
-      </c>
-      <c r="P18" s="13">
-        <f>QUARTILE(P8:P12,1)</f>
-        <v>510.53376205787782</v>
-      </c>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B19" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="14"/>
-      <c r="N19" s="13">
-        <f>MIN(N8:N12)</f>
-        <v>39.780683937823831</v>
-      </c>
-      <c r="O19" s="13">
-        <f>MIN(O8:O12)</f>
-        <v>317.57412309728659</v>
-      </c>
-      <c r="P19" s="13">
-        <f>MIN(P8:P12)</f>
-        <v>138.70038910505838</v>
-      </c>
-    </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B21" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="O21" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="P21" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B22" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J22" s="9"/>
-      <c r="N22" s="8">
-        <f>J7*N17</f>
-        <v>1108661.5028506271</v>
-      </c>
-      <c r="O22" s="8">
-        <f>K7*O17</f>
-        <v>1385111.7543648405</v>
-      </c>
-      <c r="P22" s="8">
-        <f>P24-P23</f>
-        <v>1459386.0947075211</v>
-      </c>
-    </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B23" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G23" s="1"/>
-      <c r="J23" s="9"/>
-      <c r="N23" s="8">
-        <f>G7</f>
-        <v>2176</v>
-      </c>
-      <c r="O23" s="8">
-        <f>N23</f>
-        <v>2176</v>
-      </c>
-      <c r="P23" s="8">
-        <f>G7</f>
-        <v>2176</v>
-      </c>
-    </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G24" s="1"/>
-      <c r="J24" s="9"/>
-      <c r="N24" s="8">
-        <f>N22-N23</f>
-        <v>1106485.5028506271</v>
-      </c>
-      <c r="O24" s="8">
-        <f>O22-O23</f>
-        <v>1382935.7543648405</v>
-      </c>
-      <c r="P24" s="8">
-        <f>L7*P17</f>
-        <v>1461562.0947075211</v>
-      </c>
-    </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B25" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G25" s="1"/>
-      <c r="N25" s="8">
-        <f>E7</f>
-        <v>310</v>
-      </c>
-      <c r="O25" s="8">
-        <f>N25</f>
-        <v>310</v>
-      </c>
-      <c r="P25" s="8">
-        <f>O25</f>
-        <v>310</v>
-      </c>
-    </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B26" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="3">
-        <f>N24/N25</f>
-        <v>3569.3080737117002</v>
-      </c>
-      <c r="O26" s="3">
-        <f>O24/O25</f>
-        <v>4461.0830785962598</v>
-      </c>
-      <c r="P26" s="3">
-        <f>P24/P25</f>
-        <v>4714.7164345403908</v>
-      </c>
-      <c r="Q26" s="2">
-        <f>AVERAGE(N26:P26)</f>
-        <v>4248.3691956161174</v>
-      </c>
-    </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="G27" s="1"/>
-      <c r="N27" t="str">
-        <f>IF($D$7&lt;N26,"Undervalued","Overvalued")</f>
-        <v>Undervalued</v>
-      </c>
-      <c r="O27" t="str">
-        <f>IF($D$7&lt;O26,"Undervalued","Overvalued")</f>
-        <v>Undervalued</v>
-      </c>
-      <c r="P27" t="str">
-        <f>IF($D$7&lt;P26,"Undervalued","Overvalued")</f>
-        <v>Undervalued</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="N4:P4"/>
-  </mergeCells>
-  <conditionalFormatting sqref="N27:P27">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Overvalued">
       <formula>NOT(ISERROR(SEARCH("Overvalued",N27)))</formula>
     </cfRule>

</xml_diff>